<commit_message>
fix(paper-02): 排除#79 Ding 2021，最终纳入锁定16篇
排除原因：主统计为SES分组ANOVA，MEL与SES r=0.948（共线），
父母教育无独立回归系数（composite-inseparable），E2

更新：
- 筛选表：#79改为排除E2，纳入16篇/排除93篇/合计109篇
- 提取表：删除#79行，剩16行
- Methods草稿v1.3→v1.4：16篇，E2×87
- 最终序号：#5/#7/#9/#13/#15/#19/#20/#23/#28/#43/#64/#72/#75/#78/#104/#109
- 效应方向：14正/2负

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/paper-02/03-screen/数据_5_第三轮全文筛选.xlsx
+++ b/projects/paper-02/03-screen/数据_5_第三轮全文筛选.xlsx
@@ -4792,11 +4792,19 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>纳入</t>
-        </is>
-      </c>
-      <c r="J80" s="2" t="inlineStr"/>
-      <c r="K80" s="4" t="inlineStr"/>
+          <t>排除</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>主统计为SES分组ANOVA，MEL与SES r=0.948（共线），教育无独立回归系数，composite-inseparable</t>
+        </is>
+      </c>
       <c r="L80" s="4" t="n"/>
     </row>
     <row r="81" ht="32" customHeight="1">

</xml_diff>